<commit_message>
Updated excel calculator to latest version 1.6. Fixed graphite-CO-CO2 buffer that erroneously used GPa for pressure instead of bars
</commit_message>
<xml_diff>
--- a/buffer_equations/Calc_fO2_buffer.xlsx
+++ b/buffer_equations/Calc_fO2_buffer.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="11113"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10217"/>
   <workbookPr showInkAnnotation="0" autoCompressPictures="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kiacovin/Dropbox/Research/Calculators and Spreadsheets/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kiacovino/Library/CloudStorage/Dropbox/Research/Calculators and Spreadsheets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{22F2586F-93E2-CD46-8C6E-EABDE8D04C94}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7DA16246-65E3-CE45-B93E-B408CAF9099F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="10160" yWindow="4400" windowWidth="30420" windowHeight="21000" tabRatio="678" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="11620" yWindow="3000" windowWidth="29960" windowHeight="25800" tabRatio="678" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Translate from logfO2 value" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="274" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="275" uniqueCount="71">
   <si>
     <t>Buffer</t>
   </si>
@@ -143,9 +143,6 @@
   </si>
   <si>
     <t>Graphite-CO-CO2</t>
-  </si>
-  <si>
-    <t>French and Eugster (1965)</t>
   </si>
   <si>
     <t>log(fO2) = (-20586/t) - 0.044 + log(P) - 0.028 * (P-1)/T</t>
@@ -578,10 +575,46 @@
     </r>
   </si>
   <si>
-    <t>Please cite as: Iacovino, Kayla. (2022). Calculate fO2 Buffer (1.5). Zenodo. https://doi.org/10.5281/zenodo.7387196</t>
-  </si>
-  <si>
     <t>log(fO2) = (-451020 + 297.595 * T - 14.6586T*ln(T))/(8.31441*T*ln(10))</t>
+  </si>
+  <si>
+    <t>French and Eugster (1965), P in bars</t>
+  </si>
+  <si>
+    <t>Please cite as: Iacovino, Kayla. (2026). Calculate fO2 Buffer (1.6). Zenodo. https://doi.org/10.5281/zenodo.18746164</t>
+  </si>
+  <si>
+    <r>
+      <t>Version 1.6</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color rgb="FF555555"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t> </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="16"/>
+        <color rgb="FF555555"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>23 Feb 2026</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color rgb="FF555555"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t> Fixed Graphite-CO buffer (previously converted pressure to GPa when it should have been in bars). Credit Michael Anenburg for the fix!</t>
+    </r>
   </si>
 </sst>
 </file>
@@ -591,7 +624,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="\+#0.00;\-#0.00;&quot;On Forecast&quot;"/>
   </numFmts>
-  <fonts count="12" x14ac:knownFonts="1">
+  <fonts count="13" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -678,6 +711,14 @@
       <color rgb="FF222222"/>
       <name val="Arial"/>
       <family val="2"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="16"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -882,8 +923,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="13"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="13" applyFont="1"/>
   </cellXfs>
   <cellStyles count="14">
     <cellStyle name="Followed Hyperlink" xfId="2" builtinId="9" hidden="1"/>
@@ -924,15 +965,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>7</xdr:col>
-      <xdr:colOff>495300</xdr:colOff>
-      <xdr:row>2</xdr:row>
-      <xdr:rowOff>139700</xdr:rowOff>
+      <xdr:colOff>749300</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>101600</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>14</xdr:col>
-      <xdr:colOff>749300</xdr:colOff>
-      <xdr:row>29</xdr:row>
-      <xdr:rowOff>152400</xdr:rowOff>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>177800</xdr:colOff>
+      <xdr:row>27</xdr:row>
+      <xdr:rowOff>114300</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -962,8 +1003,8 @@
       </xdr:blipFill>
       <xdr:spPr bwMode="auto">
         <a:xfrm>
-          <a:off x="6362700" y="330200"/>
-          <a:ext cx="6032500" cy="5156200"/>
+          <a:off x="6921500" y="101600"/>
+          <a:ext cx="6032500" cy="5499100"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -979,7 +1020,7 @@
         </a:ln>
         <a:extLst>
           <a:ext uri="{909E8E84-426E-40dd-AFC4-6F175D3DCCD1}">
-            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns="">
+            <a14:hiddenFill xmlns="" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
               <a:solidFill>
                 <a:srgbClr val="FFFFFF"/>
               </a:solidFill>
@@ -1408,7 +1449,7 @@
         <v>16</v>
       </c>
       <c r="C4" s="4">
-        <v>-9.9</v>
+        <v>-10.220000000000001</v>
       </c>
     </row>
     <row r="5" spans="2:6" x14ac:dyDescent="0.2">
@@ -1416,7 +1457,7 @@
         <v>18</v>
       </c>
       <c r="C5" s="6">
-        <v>1700</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="6" spans="2:6" ht="17" thickBot="1" x14ac:dyDescent="0.25">
@@ -1439,7 +1480,7 @@
       </c>
       <c r="C10">
         <f>C5+273.15</f>
-        <v>1973.15</v>
+        <v>1273.1500000000001</v>
       </c>
     </row>
     <row r="11" spans="2:6" ht="17" thickBot="1" x14ac:dyDescent="0.25"/>
@@ -1470,319 +1511,319 @@
     </row>
     <row r="14" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B14" s="18" t="s">
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="C14">
-        <f>('Equilibrium Parameters'!B3/'Translate from logfO2 value'!$C$10)+'Equilibrium Parameters'!C3+(('Equilibrium Parameters'!D3*('Translate from logfO2 value'!$C$6-1))/'Translate from logfO2 value'!$C$10)</f>
-        <v>-7.5271258393938627</v>
+        <f>('Equilibrium Parameters'!B13/'Translate from logfO2 value'!$C$10)+'Equilibrium Parameters'!C13+(('Equilibrium Parameters'!D13*('Translate from logfO2 value'!$C$6-1))/'Translate from logfO2 value'!$C$10)</f>
+        <v>-5.6970981424026998</v>
       </c>
       <c r="E14" t="s">
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="F14" s="19">
-        <f>$C$4-C14</f>
-        <v>-2.3728741606061377</v>
+        <f t="shared" ref="F14:F27" si="0">$C$4-C14</f>
+        <v>-4.5229018575973008</v>
       </c>
     </row>
     <row r="15" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B15" s="18" t="s">
-        <v>5</v>
+        <v>14</v>
       </c>
       <c r="C15">
-        <f>('Equilibrium Parameters'!B4/'Translate from logfO2 value'!$C$10)+'Equilibrium Parameters'!C4+(('Equilibrium Parameters'!D4*('Translate from logfO2 value'!$C$6-1))/'Translate from logfO2 value'!$C$10)</f>
-        <v>-7.4692548463117339</v>
+        <f>('Equilibrium Parameters'!B14/'Translate from logfO2 value'!$C$10)+'Equilibrium Parameters'!C14+(('Equilibrium Parameters'!D14*('Translate from logfO2 value'!$C$6-1))/'Translate from logfO2 value'!$C$10)</f>
+        <v>-5.322284687585908</v>
       </c>
       <c r="E15" t="s">
-        <v>5</v>
+        <v>14</v>
       </c>
       <c r="F15" s="19">
-        <f t="shared" ref="F15" si="0">$C$4-C15</f>
-        <v>-2.4307451536882665</v>
+        <f t="shared" si="0"/>
+        <v>-4.8977153124140926</v>
       </c>
     </row>
     <row r="16" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B16" s="18" t="s">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="C16">
-        <f>('Equilibrium Parameters'!B5/'Translate from logfO2 value'!$C$10)+'Equilibrium Parameters'!C5+(('Equilibrium Parameters'!D5*('Translate from logfO2 value'!$C$6-1))/'Translate from logfO2 value'!$C$10)</f>
-        <v>-7.2295308010034702</v>
+        <f>('Equilibrium Parameters'!B15/'Translate from logfO2 value'!$C$10)+'Equilibrium Parameters'!C15+(('Equilibrium Parameters'!D15*('Translate from logfO2 value'!$C$6-1))/'Translate from logfO2 value'!$C$10)</f>
+        <v>-5.6286237285473</v>
       </c>
       <c r="E16" t="s">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="F16" s="19">
-        <f t="shared" ref="F16:F32" si="1">$C$4-C16</f>
-        <v>-2.6704691989965301</v>
+        <f t="shared" si="0"/>
+        <v>-4.5913762714527007</v>
       </c>
     </row>
     <row r="17" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B17" s="18" t="s">
-        <v>29</v>
+        <v>38</v>
       </c>
       <c r="C17">
-        <f>(6.54106+0.0012324*(C6/10000)) + (-28163.6+546.32*(C6/10000)-1.13412*(C6/10000)^2+0.0019274*(C6/10000)^3)/(C5+273.15)</f>
-        <v>-7.7323328615869711</v>
+        <f>(-451020+297.595*C10-14.6586*C10*LN(C10))/(8.31441*C10*LN(10))</f>
+        <v>-8.4335986852380227</v>
       </c>
       <c r="E17" t="s">
-        <v>29</v>
+        <v>38</v>
       </c>
       <c r="F17" s="19">
-        <f t="shared" si="1"/>
-        <v>-2.1676671384130293</v>
-      </c>
-      <c r="G17" s="25" t="s">
-        <v>54</v>
+        <f t="shared" si="0"/>
+        <v>-1.7864013147619779</v>
       </c>
     </row>
     <row r="18" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B18" s="18" t="s">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="C18">
-        <f>('Equilibrium Parameters'!B7/'Translate from logfO2 value'!$C$10)+'Equilibrium Parameters'!C7+(('Equilibrium Parameters'!D7*('Translate from logfO2 value'!$C$6-1))/'Translate from logfO2 value'!$C$10)</f>
-        <v>-3.6147136304893195</v>
+        <f>('Equilibrium Parameters'!B12/'Translate from logfO2 value'!$C$10)+'Equilibrium Parameters'!C12+(('Equilibrium Parameters'!D12*('Translate from logfO2 value'!$C$6-1))/'Translate from logfO2 value'!$C$10)</f>
+        <v>-10.22135333621333</v>
       </c>
       <c r="E18" t="s">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="F18" s="19">
-        <f t="shared" si="1"/>
-        <v>-6.2852863695106809</v>
+        <f t="shared" si="0"/>
+        <v>1.3533362133291149E-3</v>
       </c>
     </row>
     <row r="19" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B19" s="18" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="C19">
-        <f>('Equilibrium Parameters'!B8/'Translate from logfO2 value'!$C$10)+'Equilibrium Parameters'!C8+(('Equilibrium Parameters'!D8*('Translate from logfO2 value'!$C$6-1))/'Translate from logfO2 value'!$C$10)</f>
-        <v>-6.4105062970377293</v>
+        <f>('Equilibrium Parameters'!B10/'Translate from logfO2 value'!$C$10)+'Equilibrium Parameters'!C10+(('Equilibrium Parameters'!D10*('Translate from logfO2 value'!$C$6-1))/'Translate from logfO2 value'!$C$10)</f>
+        <v>-10.435405411773944</v>
       </c>
       <c r="E19" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F19" s="19">
-        <f t="shared" si="1"/>
-        <v>-3.489493702962271</v>
+        <f t="shared" si="0"/>
+        <v>0.21540541177394346</v>
       </c>
     </row>
     <row r="20" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B20" s="18" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="C20">
-        <f>('Equilibrium Parameters'!B9/'Translate from logfO2 value'!$C$10)+'Equilibrium Parameters'!C9+(('Equilibrium Parameters'!D9*('Translate from logfO2 value'!$C$6-1))/'Translate from logfO2 value'!$C$10)</f>
-        <v>-5.036855155462078</v>
+        <f>('Equilibrium Parameters'!B11/'Translate from logfO2 value'!$C$10)+'Equilibrium Parameters'!C11+(('Equilibrium Parameters'!D11*('Translate from logfO2 value'!$C$6-1))/'Translate from logfO2 value'!$C$10)</f>
+        <v>-10.976974237128381</v>
       </c>
       <c r="E20" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="F20" s="19">
-        <f t="shared" si="1"/>
-        <v>-4.8631448445379224</v>
+        <f t="shared" si="0"/>
+        <v>0.75697423712838052</v>
       </c>
     </row>
     <row r="21" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B21" s="18" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C21">
-        <f>('Equilibrium Parameters'!B10/'Translate from logfO2 value'!$C$10)+'Equilibrium Parameters'!C10+(('Equilibrium Parameters'!D10*('Translate from logfO2 value'!$C$6-1))/'Translate from logfO2 value'!$C$10)</f>
-        <v>-3.0636476699693382</v>
+        <f>('Equilibrium Parameters'!B9/'Translate from logfO2 value'!$C$10)+'Equilibrium Parameters'!C9+(('Equilibrium Parameters'!D9*('Translate from logfO2 value'!$C$6-1))/'Translate from logfO2 value'!$C$10)</f>
+        <v>-11.817123473274945</v>
       </c>
       <c r="E21" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F21" s="19">
-        <f t="shared" si="1"/>
-        <v>-6.8363523300306621</v>
+        <f t="shared" si="0"/>
+        <v>1.5971234732749444</v>
       </c>
     </row>
     <row r="22" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B22" s="18" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="C22">
-        <f>('Equilibrium Parameters'!B11/'Translate from logfO2 value'!$C$10)+'Equilibrium Parameters'!C11+(('Equilibrium Parameters'!D11*('Translate from logfO2 value'!$C$6-1))/'Translate from logfO2 value'!$C$10)</f>
-        <v>-3.9839012492714687</v>
+        <f>('Equilibrium Parameters'!B7/'Translate from logfO2 value'!$C$10)+'Equilibrium Parameters'!C7+(('Equilibrium Parameters'!D7*('Translate from logfO2 value'!$C$6-1))/'Translate from logfO2 value'!$C$10)</f>
+        <v>-12.75636979146212</v>
       </c>
       <c r="E22" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="F22" s="19">
-        <f t="shared" si="1"/>
-        <v>-5.9160987507285316</v>
+        <f t="shared" si="0"/>
+        <v>2.5363697914621195</v>
       </c>
     </row>
     <row r="23" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B23" s="18" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="C23">
-        <f>('Equilibrium Parameters'!B12/'Translate from logfO2 value'!$C$10)+'Equilibrium Parameters'!C12+(('Equilibrium Parameters'!D12*('Translate from logfO2 value'!$C$6-1))/'Translate from logfO2 value'!$C$10)</f>
-        <v>-3.2746197704178606</v>
+        <f>('Equilibrium Parameters'!B8/'Translate from logfO2 value'!$C$10)+'Equilibrium Parameters'!C8+(('Equilibrium Parameters'!D8*('Translate from logfO2 value'!$C$6-1))/'Translate from logfO2 value'!$C$10)</f>
+        <v>-14.405129403448138</v>
       </c>
       <c r="E23" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="F23" s="19">
-        <f t="shared" si="1"/>
-        <v>-6.6253802295821398</v>
+        <f t="shared" si="0"/>
+        <v>4.185129403448137</v>
       </c>
     </row>
     <row r="24" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B24" s="18" t="s">
-        <v>13</v>
+        <v>46</v>
       </c>
       <c r="C24">
-        <f>('Equilibrium Parameters'!B13/'Translate from logfO2 value'!$C$10)+'Equilibrium Parameters'!C13+(('Equilibrium Parameters'!D13*('Translate from logfO2 value'!$C$6-1))/'Translate from logfO2 value'!$C$10)</f>
-        <v>1.4077690494893957</v>
+        <f>LOG(EXP((-580563+173*C10)/(8.314*C10)))</f>
+        <v>-14.783207813079107</v>
       </c>
       <c r="E24" t="s">
-        <v>13</v>
+        <v>46</v>
       </c>
       <c r="F24" s="19">
-        <f t="shared" si="1"/>
-        <v>-11.307769049489396</v>
+        <f t="shared" si="0"/>
+        <v>4.5632078130791065</v>
+      </c>
+      <c r="G24" s="25" t="s">
+        <v>52</v>
       </c>
     </row>
     <row r="25" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B25" s="18" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="C25">
-        <f>('Equilibrium Parameters'!B14/'Translate from logfO2 value'!$C$10)+'Equilibrium Parameters'!C14+(('Equilibrium Parameters'!D14*('Translate from logfO2 value'!$C$6-1))/'Translate from logfO2 value'!$C$10)</f>
-        <v>2.0487207004029102</v>
+        <f>('Equilibrium Parameters'!B5/'Translate from logfO2 value'!$C$10)+'Equilibrium Parameters'!C5+(('Equilibrium Parameters'!D5*('Translate from logfO2 value'!$C$6-1))/'Translate from logfO2 value'!$C$10)</f>
+        <v>-14.889328594431133</v>
       </c>
       <c r="E25" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="F25" s="19">
-        <f t="shared" si="1"/>
-        <v>-11.948720700402911</v>
+        <f t="shared" si="0"/>
+        <v>4.669328594431132</v>
       </c>
     </row>
     <row r="26" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B26" s="18" t="s">
-        <v>15</v>
+        <v>29</v>
       </c>
       <c r="C26">
-        <f>('Equilibrium Parameters'!B15/'Translate from logfO2 value'!$C$10)+'Equilibrium Parameters'!C15+(('Equilibrium Parameters'!D15*('Translate from logfO2 value'!$C$6-1))/'Translate from logfO2 value'!$C$10)</f>
-        <v>1.5328371892658961</v>
+        <f>(6.54106+0.0012324*(C6/10000)) + (-28163.6+546.32*(C6/10000)-1.13412*(C6/10000)^2+0.0019274*(C6/10000)^3)/(C5+273.15)</f>
+        <v>-15.580092425957922</v>
       </c>
       <c r="E26" t="s">
-        <v>15</v>
+        <v>29</v>
       </c>
       <c r="F26" s="19">
-        <f t="shared" si="1"/>
-        <v>-11.432837189265896</v>
+        <f t="shared" si="0"/>
+        <v>5.3600924259579212</v>
+      </c>
+      <c r="G26" s="25" t="s">
+        <v>53</v>
       </c>
     </row>
     <row r="27" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B27" s="18" t="s">
-        <v>28</v>
+        <v>4</v>
       </c>
       <c r="C27">
-        <f>(1/C10*0.4343*120*((0.00251*(C6/10000)^3-0.20044*(C6/10000)^2+10.32257*(C6/10000))-(0.00251*0.0001^3-0.20044*0.0001^2+10.32257*0.0001)))+(LOG(EXP((-911336+212.2423*C10-4.512*C10*LOG(C10))/(8.314*C10))))</f>
-        <v>-13.816250373453505</v>
+        <f>('Equilibrium Parameters'!B3/'Translate from logfO2 value'!$C$10)+'Equilibrium Parameters'!C3+(('Equilibrium Parameters'!D3*('Translate from logfO2 value'!$C$6-1))/'Translate from logfO2 value'!$C$10)</f>
+        <v>-15.729370734006205</v>
       </c>
       <c r="E27" t="s">
-        <v>28</v>
+        <v>4</v>
       </c>
       <c r="F27" s="19">
-        <f t="shared" si="1"/>
-        <v>3.9162503734535044</v>
+        <f t="shared" si="0"/>
+        <v>5.5093707340062039</v>
       </c>
     </row>
     <row r="28" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B28" s="18" t="s">
-        <v>33</v>
+        <v>5</v>
       </c>
       <c r="C28">
-        <f>(-20586/C10) - 0.044 +LOG10(C6/10000) - 0.028 * ((C6/10000)-1)/C10</f>
-        <v>-14.477049693535717</v>
+        <f>('Equilibrium Parameters'!B4/'Translate from logfO2 value'!$C$10)+'Equilibrium Parameters'!C4+(('Equilibrium Parameters'!D4*('Translate from logfO2 value'!$C$6-1))/'Translate from logfO2 value'!$C$10)</f>
+        <v>-15.695212818599533</v>
       </c>
       <c r="E28" t="s">
-        <v>33</v>
+        <v>5</v>
       </c>
       <c r="F28" s="19">
-        <f t="shared" si="1"/>
-        <v>4.5770496935357166</v>
+        <f t="shared" ref="F28" si="1">$C$4-C28</f>
+        <v>5.4752128185995321</v>
       </c>
     </row>
     <row r="29" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B29" s="18" t="s">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="C29">
-        <f>(-451020+297.595*C10-14.6586*C10*LN(C10))/(8.31441*C10*LN(10))</f>
-        <v>-2.2044885917095569</v>
+        <f>(-20586/C10) - 0.044 +LOG10(C6) - 0.028 * ((C6)-1)/C10</f>
+        <v>-16.213343753681812</v>
       </c>
       <c r="E29" t="s">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="F29" s="19">
-        <f t="shared" si="1"/>
-        <v>-7.695511408290443</v>
+        <f t="shared" ref="F29" si="2">$C$4-C29</f>
+        <v>5.9933437536818115</v>
       </c>
     </row>
     <row r="30" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B30" s="18" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C30">
         <f>LOG(EXP((-758585+349.718*C10-25.5216*C10*LN(C10)+0.00935*C10^2)/(8.314*C10)))</f>
-        <v>-10.965966159078675</v>
+        <v>-21.765471947809271</v>
       </c>
       <c r="E30" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="F30" s="19">
-        <f t="shared" si="1"/>
-        <v>1.0659661590786751</v>
+        <f>$C$4-C30</f>
+        <v>11.54547194780927</v>
       </c>
       <c r="G30" s="25" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="31" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B31" s="18" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="C31">
-        <f>LOG(EXP((-580563+173*C10)/(8.314*C10)))</f>
-        <v>-6.3327155358643328</v>
+        <f>2*LOG(EXP((-376969-4.19123*C10+10.02409*C10*LN(C10))/(8.314*C10)))</f>
+        <v>-23.884430305504146</v>
       </c>
       <c r="E31" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="F31" s="19">
-        <f t="shared" si="1"/>
-        <v>-3.5672844641356676</v>
+        <f>$C$4-C31</f>
+        <v>13.664430305504146</v>
       </c>
       <c r="G31" s="25" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="32" spans="2:7" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B32" s="20" t="s">
-        <v>50</v>
+        <v>28</v>
       </c>
       <c r="C32" s="21">
-        <f>2*LOG(EXP((-376969-4.19123*C10+10.02409*C10*LN(C10))/(8.314*C10)))</f>
-        <v>-12.451508207938426</v>
+        <f>(1/C10*0.4343*120*((0.00251*(C6/10000)^3-0.20044*(C6/10000)^2+10.32257*(C6/10000))-(0.00251*0.0001^3-0.20044*0.0001^2+10.32257*0.0001)))+(LOG(EXP((-911336+212.2423*C10-4.512*C10*LOG(C10))/(8.314*C10))))</f>
+        <v>-27.036522869930032</v>
       </c>
       <c r="D32" s="21"/>
       <c r="E32" s="21" t="s">
-        <v>50</v>
+        <v>28</v>
       </c>
       <c r="F32" s="22">
-        <f t="shared" si="1"/>
-        <v>2.5515082079384257</v>
-      </c>
-      <c r="G32" s="25" t="s">
-        <v>53</v>
+        <f>$C$4-C32</f>
+        <v>16.816522869930033</v>
       </c>
     </row>
   </sheetData>
@@ -1812,7 +1853,7 @@
         <v>25</v>
       </c>
       <c r="C4" s="4">
-        <v>-5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5" spans="2:6" x14ac:dyDescent="0.2">
@@ -1820,7 +1861,7 @@
         <v>18</v>
       </c>
       <c r="C5" s="6">
-        <v>1400</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="6" spans="2:6" ht="17" thickBot="1" x14ac:dyDescent="0.25">
@@ -1842,8 +1883,8 @@
         <v>26</v>
       </c>
       <c r="C10" s="13">
-        <f>C24+C4</f>
-        <v>-11.264432208708124</v>
+        <f>C22+C4</f>
+        <v>-10.976974237128381</v>
       </c>
       <c r="D10" s="13"/>
       <c r="E10" s="13"/>
@@ -1859,7 +1900,7 @@
       </c>
       <c r="C12">
         <f>C5+273.15</f>
-        <v>1673.15</v>
+        <v>1273.1500000000001</v>
       </c>
       <c r="F12" s="24"/>
     </row>
@@ -1892,319 +1933,319 @@
     </row>
     <row r="16" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B16" s="18" t="s">
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="C16">
-        <f>('Equilibrium Parameters'!B3/$C$12)+'Equilibrium Parameters'!C3+(('Equilibrium Parameters'!D3*($C$6-1))/C$12)</f>
-        <v>-10.201983294982517</v>
+        <f>('Equilibrium Parameters'!B13/$C$12)+'Equilibrium Parameters'!C13+(('Equilibrium Parameters'!D13*($C$6-1))/C$12)</f>
+        <v>-5.6970981424026998</v>
       </c>
       <c r="E16" t="s">
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="F16" s="19">
-        <f>$C$10-C16</f>
-        <v>-1.062448913725607</v>
+        <f t="shared" ref="F16:F29" si="0">$C$10-C16</f>
+        <v>-5.2798760947256813</v>
       </c>
     </row>
     <row r="17" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B17" s="18" t="s">
-        <v>5</v>
+        <v>14</v>
       </c>
       <c r="C17">
-        <f>('Equilibrium Parameters'!B4/$C$12)+'Equilibrium Parameters'!C4+(('Equilibrium Parameters'!D4*($C$6-1))/C$12)</f>
-        <v>-10.151845441233601</v>
+        <f>('Equilibrium Parameters'!B14/$C$12)+'Equilibrium Parameters'!C14+(('Equilibrium Parameters'!D14*($C$6-1))/C$12)</f>
+        <v>-5.322284687585908</v>
       </c>
       <c r="E17" t="s">
-        <v>5</v>
+        <v>14</v>
       </c>
       <c r="F17" s="19">
-        <f t="shared" ref="F17:F32" si="0">$C$10-C17</f>
-        <v>-1.1125867674745233</v>
+        <f t="shared" si="0"/>
+        <v>-5.6546895495424732</v>
       </c>
     </row>
     <row r="18" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B18" s="18" t="s">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="C18">
-        <f>('Equilibrium Parameters'!B5/$C$12)+'Equilibrium Parameters'!C5+(('Equilibrium Parameters'!D5*($C$6-1))/C$12)</f>
-        <v>-9.7274892866748335</v>
+        <f>('Equilibrium Parameters'!B15/$C$12)+'Equilibrium Parameters'!C15+(('Equilibrium Parameters'!D15*($C$6-1))/C$12)</f>
+        <v>-5.6286237285473</v>
       </c>
       <c r="E18" t="s">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="F18" s="19">
         <f t="shared" si="0"/>
-        <v>-1.5369429220332904</v>
+        <v>-5.3483505085810812</v>
       </c>
     </row>
     <row r="19" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B19" s="18" t="s">
-        <v>29</v>
+        <v>38</v>
       </c>
       <c r="C19">
-        <f>(6.54106+0.0012324*(C6/10000)) + (-28163.6+546.32*(C6/10000)-1.13412*(C6/10000)^2+0.0019274*(C6/10000)^3)/(C5+273.15)</f>
-        <v>-10.29158809599398</v>
+        <f>(-451020+297.595*C12-14.6586*C12*LN(C12))/(8.31441*C12*LN(10))</f>
+        <v>-8.4335986852380227</v>
       </c>
       <c r="E19" t="s">
-        <v>29</v>
+        <v>38</v>
       </c>
       <c r="F19" s="19">
-        <f>$C$10-C19</f>
-        <v>-0.97284411271414406</v>
-      </c>
-      <c r="G19" s="25" t="s">
-        <v>54</v>
+        <f t="shared" si="0"/>
+        <v>-2.5433755518903585</v>
       </c>
     </row>
     <row r="20" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B20" s="18" t="s">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="C20">
-        <f>('Equilibrium Parameters'!B7/$C$12)+'Equilibrium Parameters'!C7+(('Equilibrium Parameters'!D7*($C$6-1))/C$12)</f>
-        <v>-6.5959251710844811</v>
+        <f>('Equilibrium Parameters'!B12/$C$12)+'Equilibrium Parameters'!C12+(('Equilibrium Parameters'!D12*($C$6-1))/C$12)</f>
+        <v>-10.22135333621333</v>
       </c>
       <c r="E20" t="s">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="F20" s="19">
         <f t="shared" si="0"/>
-        <v>-4.6685070376236428</v>
+        <v>-0.75562090091505141</v>
       </c>
     </row>
     <row r="21" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B21" s="18" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="C21">
-        <f>('Equilibrium Parameters'!B8/$C$12)+'Equilibrium Parameters'!C8+(('Equilibrium Parameters'!D8*($C$6-1))/C$12)</f>
-        <v>-9.0176556196395996</v>
+        <f>('Equilibrium Parameters'!B10/$C$12)+'Equilibrium Parameters'!C10+(('Equilibrium Parameters'!D10*($C$6-1))/C$12)</f>
+        <v>-10.435405411773944</v>
       </c>
       <c r="E21" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F21" s="19">
         <f t="shared" si="0"/>
-        <v>-2.2467765890685243</v>
+        <v>-0.54156882535443707</v>
       </c>
     </row>
     <row r="22" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B22" s="18" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="C22">
-        <f>('Equilibrium Parameters'!B9/$C$12)+'Equilibrium Parameters'!C9+(('Equilibrium Parameters'!D9*($C$6-1))/C$12)</f>
-        <v>-7.2479877775453474</v>
+        <f>('Equilibrium Parameters'!B11/$C$12)+'Equilibrium Parameters'!C11+(('Equilibrium Parameters'!D11*($C$6-1))/C$12)</f>
+        <v>-10.976974237128381</v>
       </c>
       <c r="E22" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="F22" s="19">
         <f t="shared" si="0"/>
-        <v>-4.0164444311627765</v>
+        <v>0</v>
       </c>
     </row>
     <row r="23" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B23" s="18" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C23">
-        <f>('Equilibrium Parameters'!B10/$C$12)+'Equilibrium Parameters'!C10+(('Equilibrium Parameters'!D10*($C$6-1))/C$12)</f>
-        <v>-5.4676725936108532</v>
+        <f>('Equilibrium Parameters'!B9/$C$12)+'Equilibrium Parameters'!C9+(('Equilibrium Parameters'!D9*($C$6-1))/C$12)</f>
+        <v>-11.817123473274945</v>
       </c>
       <c r="E23" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F23" s="19">
         <f t="shared" si="0"/>
-        <v>-5.7967596150972707</v>
+        <v>0.84014923614656389</v>
       </c>
     </row>
     <row r="24" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B24" s="18" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="C24">
-        <f>('Equilibrium Parameters'!B11/$C$12)+'Equilibrium Parameters'!C11+(('Equilibrium Parameters'!D11*($C$6-1))/C$12)</f>
-        <v>-6.2644322087081239</v>
+        <f>('Equilibrium Parameters'!B7/$C$12)+'Equilibrium Parameters'!C7+(('Equilibrium Parameters'!D7*($C$6-1))/C$12)</f>
+        <v>-12.75636979146212</v>
       </c>
       <c r="E24" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="F24" s="19">
         <f t="shared" si="0"/>
-        <v>-5</v>
+        <v>1.779395554333739</v>
       </c>
     </row>
     <row r="25" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B25" s="18" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="C25">
-        <f>('Equilibrium Parameters'!B12/$C$12)+'Equilibrium Parameters'!C12+(('Equilibrium Parameters'!D12*($C$6-1))/C$12)</f>
-        <v>-5.5400388488778649</v>
+        <f>('Equilibrium Parameters'!B8/$C$12)+'Equilibrium Parameters'!C8+(('Equilibrium Parameters'!D8*($C$6-1))/C$12)</f>
+        <v>-14.405129403448138</v>
       </c>
       <c r="E25" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="F25" s="19">
         <f t="shared" si="0"/>
-        <v>-5.724393359830259</v>
+        <v>3.4281551663197565</v>
       </c>
     </row>
     <row r="26" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B26" s="18" t="s">
-        <v>13</v>
+        <v>46</v>
       </c>
       <c r="C26">
-        <f>('Equilibrium Parameters'!B13/$C$12)+'Equilibrium Parameters'!C13+(('Equilibrium Parameters'!D13*($C$6-1))/C$12)</f>
-        <v>-0.90921943639243175</v>
+        <f>LOG(EXP((-580563+173*C12)/(8.314*C12)))</f>
+        <v>-14.783207813079107</v>
       </c>
       <c r="E26" t="s">
-        <v>13</v>
+        <v>46</v>
       </c>
       <c r="F26" s="19">
         <f t="shared" si="0"/>
-        <v>-10.355212772315692</v>
+        <v>3.806233575950726</v>
+      </c>
+      <c r="G26" s="25" t="s">
+        <v>52</v>
       </c>
     </row>
     <row r="27" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B27" s="18" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="C27">
-        <f>('Equilibrium Parameters'!B14/$C$12)+'Equilibrium Parameters'!C14+(('Equilibrium Parameters'!D14*($C$6-1))/C$12)</f>
-        <v>-0.35505887099184008</v>
+        <f>('Equilibrium Parameters'!B5/$C$12)+'Equilibrium Parameters'!C5+(('Equilibrium Parameters'!D5*($C$6-1))/C$12)</f>
+        <v>-14.889328594431133</v>
       </c>
       <c r="E27" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="F27" s="19">
         <f t="shared" si="0"/>
-        <v>-10.909373337716284</v>
+        <v>3.9123543573027515</v>
       </c>
     </row>
     <row r="28" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B28" s="18" t="s">
-        <v>15</v>
+        <v>29</v>
       </c>
       <c r="C28">
-        <f>('Equilibrium Parameters'!B15/$C$12)+'Equilibrium Parameters'!C15+(('Equilibrium Parameters'!D15*($C$6-1))/C$12)</f>
-        <v>-0.80260723784478216</v>
+        <f>(6.54106+0.0012324*(C6/10000)) + (-28163.6+546.32*(C6/10000)-1.13412*(C6/10000)^2+0.0019274*(C6/10000)^3)/(C5+273.15)</f>
+        <v>-15.580092425957922</v>
       </c>
       <c r="E28" t="s">
-        <v>15</v>
+        <v>29</v>
       </c>
       <c r="F28" s="19">
         <f t="shared" si="0"/>
-        <v>-10.461824970863342</v>
+        <v>4.6031181888295407</v>
+      </c>
+      <c r="G28" s="25" t="s">
+        <v>53</v>
       </c>
     </row>
     <row r="29" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B29" s="18" t="s">
-        <v>28</v>
+        <v>4</v>
       </c>
       <c r="C29">
-        <f>(1/C12*0.4343*120*((0.00251*(C6/10000)^3-0.20044*(C6/10000)^2+10.32257*(C6/10000))-(0.00251*0.0001^3-0.20044*0.0001^2+10.32257*0.0001)))+(LOG(EXP((-911336+212.2423*C12-4.512*C12*LOG(C12))/(8.314*C12))))</f>
-        <v>-18.125295002865954</v>
+        <f>('Equilibrium Parameters'!B3/$C$12)+'Equilibrium Parameters'!C3+(('Equilibrium Parameters'!D3*($C$6-1))/C$12)</f>
+        <v>-15.729370734006205</v>
       </c>
       <c r="E29" t="s">
-        <v>28</v>
+        <v>4</v>
       </c>
       <c r="F29" s="19">
         <f t="shared" si="0"/>
-        <v>6.8608627941578302</v>
+        <v>4.7523964968778234</v>
       </c>
     </row>
     <row r="30" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B30" s="18" t="s">
-        <v>33</v>
+        <v>5</v>
       </c>
       <c r="C30">
-        <f>(-20586/C12) - 0.044 +LOG10(C6/10000) - 0.028 * ((C6/10000)-1)/C12</f>
-        <v>-16.347721724172963</v>
+        <f>('Equilibrium Parameters'!B4/$C$12)+'Equilibrium Parameters'!C4+(('Equilibrium Parameters'!D4*($C$6-1))/C$12)</f>
+        <v>-15.695212818599533</v>
       </c>
       <c r="E30" t="s">
-        <v>33</v>
+        <v>5</v>
       </c>
       <c r="F30" s="19">
-        <f t="shared" si="0"/>
-        <v>5.0832895154648394</v>
+        <f t="shared" ref="F30:F32" si="1">$C$10-C30</f>
+        <v>4.7182385814711516</v>
       </c>
     </row>
     <row r="31" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B31" s="18" t="s">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="C31">
-        <f>(-451020+297.595*C12-14.6586*C12*LN(C12))/(8.31441*C12*LN(10))</f>
-        <v>-4.2190051316565533</v>
+        <f>(-20586/C12) - 0.044 +LOG10(C6) - 0.028 * ((C6)-1)/C12</f>
+        <v>-16.213343753681812</v>
       </c>
       <c r="E31" t="s">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="F31" s="19">
-        <f t="shared" si="0"/>
-        <v>-7.0454270770515706</v>
+        <f t="shared" si="1"/>
+        <v>5.236369516553431</v>
       </c>
     </row>
     <row r="32" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B32" s="18" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C32">
         <f>LOG(EXP((-758585+349.718*C12-25.5216*C12*LN(C12)+0.00935*C12^2)/(8.314*C12)))</f>
-        <v>-14.493468913562438</v>
+        <v>-21.765471947809271</v>
       </c>
       <c r="E32" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="F32" s="19">
-        <f t="shared" si="0"/>
-        <v>3.2290367048543143</v>
+        <f t="shared" si="1"/>
+        <v>10.78849771068089</v>
       </c>
       <c r="G32" s="25" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="33" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B33" s="18" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="C33">
-        <f>LOG(EXP((-580563+173*C12)/(8.314*C12)))</f>
-        <v>-9.0885296527958683</v>
+        <f>2*LOG(EXP((-376969-4.19123*C12+10.02409*C12*LN(C12))/(8.314*C12)))</f>
+        <v>-23.884430305504146</v>
       </c>
       <c r="E33" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="F33" s="19">
         <f>$C$10-C33</f>
-        <v>-2.1759025559122556</v>
+        <v>12.907456068375765</v>
       </c>
       <c r="G33" s="25" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="34" spans="2:7" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B34" s="20" t="s">
-        <v>50</v>
+        <v>28</v>
       </c>
       <c r="C34" s="21">
-        <f>2*LOG(EXP((-376969-4.19123*C12+10.02409*C12*LN(C12))/(8.314*C12)))</f>
-        <v>-16.203013424383567</v>
+        <f>(1/C12*0.4343*120*((0.00251*(C6/10000)^3-0.20044*(C6/10000)^2+10.32257*(C6/10000))-(0.00251*0.0001^3-0.20044*0.0001^2+10.32257*0.0001)))+(LOG(EXP((-911336+212.2423*C12-4.512*C12*LOG(C12))/(8.314*C12))))</f>
+        <v>-27.036522869930032</v>
       </c>
       <c r="D34" s="21"/>
       <c r="E34" s="21" t="s">
-        <v>50</v>
+        <v>28</v>
       </c>
       <c r="F34" s="22">
         <f>$C$10-C34</f>
-        <v>4.9385812156754429</v>
-      </c>
-      <c r="G34" s="25" t="s">
-        <v>53</v>
+        <v>16.059548632801651</v>
       </c>
     </row>
   </sheetData>
@@ -2242,7 +2283,7 @@
         <v>18</v>
       </c>
       <c r="C5" s="6">
-        <v>750</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="6" spans="2:6" ht="17" thickBot="1" x14ac:dyDescent="0.25">
@@ -2250,7 +2291,7 @@
         <v>22</v>
       </c>
       <c r="C6" s="2">
-        <v>20812.717000000001</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7" spans="2:6" ht="17" thickTop="1" x14ac:dyDescent="0.2"/>
@@ -2264,8 +2305,8 @@
         <v>26</v>
       </c>
       <c r="C10" s="13">
-        <f>C25+C4</f>
-        <v>-14.070250713971559</v>
+        <f>C20+C4</f>
+        <v>-10.22135333621333</v>
       </c>
       <c r="D10" s="13"/>
       <c r="E10" s="13"/>
@@ -2281,7 +2322,7 @@
       </c>
       <c r="C12">
         <f>C5+273.15</f>
-        <v>1023.15</v>
+        <v>1273.1500000000001</v>
       </c>
       <c r="F12" s="24"/>
     </row>
@@ -2314,319 +2355,319 @@
     </row>
     <row r="16" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B16" s="18" t="s">
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="C16">
-        <f>('Equilibrium Parameters'!B3/$C$12)+'Equilibrium Parameters'!C3+(('Equilibrium Parameters'!D3*($C$6-1))/C$12)</f>
-        <v>-20.483685483066999</v>
+        <f>('Equilibrium Parameters'!B13/$C$12)+'Equilibrium Parameters'!C13+(('Equilibrium Parameters'!D13*($C$6-1))/C$12)</f>
+        <v>-5.6970981424026998</v>
       </c>
       <c r="E16" t="s">
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="F16" s="19">
-        <f>$C$10-C16</f>
-        <v>6.4134347690954403</v>
+        <f t="shared" ref="F16:F29" si="0">$C$10-C16</f>
+        <v>-4.5242551938106299</v>
       </c>
     </row>
     <row r="17" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B17" s="18" t="s">
-        <v>5</v>
+        <v>14</v>
       </c>
       <c r="C17">
-        <f>('Equilibrium Parameters'!B4/$C$12)+'Equilibrium Parameters'!C4+(('Equilibrium Parameters'!D4*($C$6-1))/C$12)</f>
-        <v>-20.34381503200899</v>
+        <f>('Equilibrium Parameters'!B14/$C$12)+'Equilibrium Parameters'!C14+(('Equilibrium Parameters'!D14*($C$6-1))/C$12)</f>
+        <v>-5.322284687585908</v>
       </c>
       <c r="E17" t="s">
-        <v>5</v>
+        <v>14</v>
       </c>
       <c r="F17" s="19">
-        <f t="shared" ref="F17:F32" si="0">$C$10-C17</f>
-        <v>6.2735643180374314</v>
+        <f t="shared" si="0"/>
+        <v>-4.8990686486274218</v>
       </c>
     </row>
     <row r="18" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B18" s="18" t="s">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="C18">
-        <f>('Equilibrium Parameters'!B5/$C$12)+'Equilibrium Parameters'!C5+(('Equilibrium Parameters'!D5*($C$6-1))/C$12)</f>
-        <v>-19.046282817768656</v>
+        <f>('Equilibrium Parameters'!B15/$C$12)+'Equilibrium Parameters'!C15+(('Equilibrium Parameters'!D15*($C$6-1))/C$12)</f>
+        <v>-5.6286237285473</v>
       </c>
       <c r="E18" t="s">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="F18" s="19">
         <f t="shared" si="0"/>
-        <v>4.9760321037970972</v>
+        <v>-4.5927296076660298</v>
       </c>
     </row>
     <row r="19" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B19" s="18" t="s">
-        <v>29</v>
+        <v>38</v>
       </c>
       <c r="C19">
-        <f>(6.54106+0.0012324*(C6/10000)) + (-28163.6+546.32*(C6/10000)-1.13412*(C6/10000)^2+0.0019274*(C6/10000)^3)/(C5+273.15)</f>
-        <v>-19.876210770538453</v>
+        <f>(-451020+297.595*C12-14.6586*C12*LN(C12))/(8.31441*C12*LN(10))</f>
+        <v>-8.4335986852380227</v>
       </c>
       <c r="E19" t="s">
-        <v>29</v>
+        <v>38</v>
       </c>
       <c r="F19" s="19">
-        <f>$C$10-C19</f>
-        <v>5.8059600565668941</v>
-      </c>
-      <c r="G19" s="25" t="s">
-        <v>54</v>
+        <f t="shared" si="0"/>
+        <v>-1.7877546509753071</v>
       </c>
     </row>
     <row r="20" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B20" s="18" t="s">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="C20">
-        <f>('Equilibrium Parameters'!B7/$C$12)+'Equilibrium Parameters'!C7+(('Equilibrium Parameters'!D7*($C$6-1))/C$12)</f>
-        <v>-17.364413516102232</v>
+        <f>('Equilibrium Parameters'!B12/$C$12)+'Equilibrium Parameters'!C12+(('Equilibrium Parameters'!D12*($C$6-1))/C$12)</f>
+        <v>-10.22135333621333</v>
       </c>
       <c r="E20" t="s">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="F20" s="19">
         <f t="shared" si="0"/>
-        <v>3.294162802130673</v>
+        <v>0</v>
       </c>
     </row>
     <row r="21" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B21" s="18" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="C21">
-        <f>('Equilibrium Parameters'!B8/$C$12)+'Equilibrium Parameters'!C8+(('Equilibrium Parameters'!D8*($C$6-1))/C$12)</f>
-        <v>-18.772354344915207</v>
+        <f>('Equilibrium Parameters'!B10/$C$12)+'Equilibrium Parameters'!C10+(('Equilibrium Parameters'!D10*($C$6-1))/C$12)</f>
+        <v>-10.435405411773944</v>
       </c>
       <c r="E21" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F21" s="19">
         <f t="shared" si="0"/>
-        <v>4.7021036309436486</v>
+        <v>0.21405207556061434</v>
       </c>
     </row>
     <row r="22" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B22" s="18" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="C22">
-        <f>('Equilibrium Parameters'!B9/$C$12)+'Equilibrium Parameters'!C9+(('Equilibrium Parameters'!D9*($C$6-1))/C$12)</f>
-        <v>-15.429322646728243</v>
+        <f>('Equilibrium Parameters'!B11/$C$12)+'Equilibrium Parameters'!C11+(('Equilibrium Parameters'!D11*($C$6-1))/C$12)</f>
+        <v>-10.976974237128381</v>
       </c>
       <c r="E22" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="F22" s="19">
         <f t="shared" si="0"/>
-        <v>1.3590719327566845</v>
+        <v>0.75562090091505141</v>
       </c>
     </row>
     <row r="23" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B23" s="18" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C23">
-        <f>('Equilibrium Parameters'!B10/$C$12)+'Equilibrium Parameters'!C10+(('Equilibrium Parameters'!D10*($C$6-1))/C$12)</f>
-        <v>-13.641360930459854</v>
+        <f>('Equilibrium Parameters'!B9/$C$12)+'Equilibrium Parameters'!C9+(('Equilibrium Parameters'!D9*($C$6-1))/C$12)</f>
+        <v>-11.817123473274945</v>
       </c>
       <c r="E23" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F23" s="19">
         <f t="shared" si="0"/>
-        <v>-0.42888978351170515</v>
+        <v>1.5957701370616153</v>
       </c>
     </row>
     <row r="24" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B24" s="18" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="C24">
-        <f>('Equilibrium Parameters'!B11/$C$12)+'Equilibrium Parameters'!C11+(('Equilibrium Parameters'!D11*($C$6-1))/C$12)</f>
-        <v>-13.55597505742071</v>
+        <f>('Equilibrium Parameters'!B7/$C$12)+'Equilibrium Parameters'!C7+(('Equilibrium Parameters'!D7*($C$6-1))/C$12)</f>
+        <v>-12.75636979146212</v>
       </c>
       <c r="E24" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="F24" s="19">
         <f t="shared" si="0"/>
-        <v>-0.51427565655084884</v>
+        <v>2.5350164552487904</v>
       </c>
     </row>
     <row r="25" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B25" s="18" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="C25">
-        <f>('Equilibrium Parameters'!B12/$C$12)+'Equilibrium Parameters'!C12+(('Equilibrium Parameters'!D12*($C$6-1))/C$12)</f>
-        <v>-14.070250713971559</v>
+        <f>('Equilibrium Parameters'!B8/$C$12)+'Equilibrium Parameters'!C8+(('Equilibrium Parameters'!D8*($C$6-1))/C$12)</f>
+        <v>-14.405129403448138</v>
       </c>
       <c r="E25" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="F25" s="19">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>4.1837760672348079</v>
       </c>
     </row>
     <row r="26" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B26" s="18" t="s">
-        <v>13</v>
+        <v>46</v>
       </c>
       <c r="C26">
-        <f>('Equilibrium Parameters'!B13/$C$12)+'Equilibrium Parameters'!C13+(('Equilibrium Parameters'!D13*($C$6-1))/C$12)</f>
-        <v>-10.204112668719153</v>
+        <f>LOG(EXP((-580563+173*C12)/(8.314*C12)))</f>
+        <v>-14.783207813079107</v>
       </c>
       <c r="E26" t="s">
-        <v>13</v>
+        <v>46</v>
       </c>
       <c r="F26" s="19">
         <f t="shared" si="0"/>
-        <v>-3.8661380452524057</v>
+        <v>4.5618544768657774</v>
+      </c>
+      <c r="G26" s="25" t="s">
+        <v>52</v>
       </c>
     </row>
     <row r="27" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B27" s="18" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="C27">
-        <f>('Equilibrium Parameters'!B14/$C$12)+'Equilibrium Parameters'!C14+(('Equilibrium Parameters'!D14*($C$6-1))/C$12)</f>
-        <v>-10.01260238185994</v>
+        <f>('Equilibrium Parameters'!B5/$C$12)+'Equilibrium Parameters'!C5+(('Equilibrium Parameters'!D5*($C$6-1))/C$12)</f>
+        <v>-14.889328594431133</v>
       </c>
       <c r="E27" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="F27" s="19">
         <f t="shared" si="0"/>
-        <v>-4.0576483321116186</v>
+        <v>4.6679752582178029</v>
       </c>
     </row>
     <row r="28" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B28" s="18" t="s">
-        <v>15</v>
+        <v>29</v>
       </c>
       <c r="C28">
-        <f>('Equilibrium Parameters'!B15/$C$12)+'Equilibrium Parameters'!C15+(('Equilibrium Parameters'!D15*($C$6-1))/C$12)</f>
-        <v>-10.174617286810339</v>
+        <f>(6.54106+0.0012324*(C6/10000)) + (-28163.6+546.32*(C6/10000)-1.13412*(C6/10000)^2+0.0019274*(C6/10000)^3)/(C5+273.15)</f>
+        <v>-15.580092425957922</v>
       </c>
       <c r="E28" t="s">
-        <v>15</v>
+        <v>29</v>
       </c>
       <c r="F28" s="19">
         <f t="shared" si="0"/>
-        <v>-3.8956334271612203</v>
+        <v>5.3587390897445921</v>
+      </c>
+      <c r="G28" s="25" t="s">
+        <v>53</v>
       </c>
     </row>
     <row r="29" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B29" s="18" t="s">
-        <v>28</v>
+        <v>4</v>
       </c>
       <c r="C29">
-        <f>(1/C12*0.4343*120*((0.00251*(C6/10000)^3-0.20044*(C6/10000)^2+10.32257*(C6/10000))-(0.00251*0.0001^3-0.20044*0.0001^2+10.32257*0.0001)))+(LOG(EXP((-911336+212.2423*C12-4.512*C12*LOG(C12))/(8.314*C12))))</f>
-        <v>-35.099317187436306</v>
+        <f>('Equilibrium Parameters'!B3/$C$12)+'Equilibrium Parameters'!C3+(('Equilibrium Parameters'!D3*($C$6-1))/C$12)</f>
+        <v>-15.729370734006205</v>
       </c>
       <c r="E29" t="s">
-        <v>28</v>
+        <v>4</v>
       </c>
       <c r="F29" s="19">
         <f t="shared" si="0"/>
-        <v>21.029066473464745</v>
+        <v>5.5080173977928748</v>
       </c>
     </row>
     <row r="30" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B30" s="18" t="s">
-        <v>33</v>
+        <v>5</v>
       </c>
       <c r="C30">
-        <f>(-20586/C12) - 0.044 +LOG10(C6/10000) - 0.028 * ((C6/10000)-1)/C12</f>
-        <v>-19.84591778860214</v>
+        <f>('Equilibrium Parameters'!B4/$C$12)+'Equilibrium Parameters'!C4+(('Equilibrium Parameters'!D4*($C$6-1))/C$12)</f>
+        <v>-15.695212818599533</v>
       </c>
       <c r="E30" t="s">
-        <v>33</v>
+        <v>5</v>
       </c>
       <c r="F30" s="19">
-        <f t="shared" si="0"/>
-        <v>5.7756670746305812</v>
+        <f t="shared" ref="F30:F32" si="1">$C$10-C30</f>
+        <v>5.473859482386203</v>
       </c>
     </row>
     <row r="31" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B31" s="18" t="s">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="C31">
-        <f>(-451020+297.595*C12-14.6586*C12*LN(C12))/(8.31441*C12*LN(10))</f>
-        <v>-12.787583051012373</v>
+        <f>(-20586/C12) - 0.044 +LOG10(C6) - 0.028 * ((C6)-1)/C12</f>
+        <v>-16.213343753681812</v>
       </c>
       <c r="E31" t="s">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="F31" s="19">
-        <f t="shared" si="0"/>
-        <v>-1.2826676629591862</v>
+        <f t="shared" si="1"/>
+        <v>5.9919904174684824</v>
       </c>
     </row>
     <row r="32" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B32" s="18" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C32">
         <f>LOG(EXP((-758585+349.718*C12-25.5216*C12*LN(C12)+0.00935*C12^2)/(8.314*C12)))</f>
-        <v>-29.201143258581439</v>
+        <v>-21.765471947809271</v>
       </c>
       <c r="E32" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="F32" s="19">
-        <f t="shared" si="0"/>
-        <v>15.13089254460988</v>
+        <f t="shared" si="1"/>
+        <v>11.544118611595941</v>
       </c>
       <c r="G32" s="25" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="33" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B33" s="18" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="C33">
-        <f>LOG(EXP((-580563+173*C12)/(8.314*C12)))</f>
-        <v>-20.603499781435357</v>
+        <f>2*LOG(EXP((-376969-4.19123*C12+10.02409*C12*LN(C12))/(8.314*C12)))</f>
+        <v>-23.884430305504146</v>
       </c>
       <c r="E33" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="F33" s="19">
         <f>$C$10-C33</f>
-        <v>6.5332490674637977</v>
+        <v>13.663076969290817</v>
       </c>
       <c r="G33" s="25" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="34" spans="2:7" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B34" s="20" t="s">
-        <v>50</v>
+        <v>28</v>
       </c>
       <c r="C34" s="21">
-        <f>2*LOG(EXP((-376969-4.19123*C12+10.02409*C12*LN(C12))/(8.314*C12)))</f>
-        <v>-31.67178749226445</v>
+        <f>(1/C12*0.4343*120*((0.00251*(C6/10000)^3-0.20044*(C6/10000)^2+10.32257*(C6/10000))-(0.00251*0.0001^3-0.20044*0.0001^2+10.32257*0.0001)))+(LOG(EXP((-911336+212.2423*C12-4.512*C12*LOG(C12))/(8.314*C12))))</f>
+        <v>-27.036522869930032</v>
       </c>
       <c r="D34" s="21"/>
       <c r="E34" s="21" t="s">
-        <v>50</v>
+        <v>28</v>
       </c>
       <c r="F34" s="22">
         <f>$C$10-C34</f>
-        <v>17.601536778292889</v>
-      </c>
-      <c r="G34" s="25" t="s">
-        <v>53</v>
+        <v>16.815169533716702</v>
       </c>
     </row>
   </sheetData>
@@ -2651,10 +2692,10 @@
     </row>
     <row r="4" spans="2:6" ht="17" thickTop="1" x14ac:dyDescent="0.2">
       <c r="B4" s="11" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C4" s="4">
-        <v>-5.05</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5" spans="2:6" x14ac:dyDescent="0.2">
@@ -2662,7 +2703,7 @@
         <v>18</v>
       </c>
       <c r="C5" s="6">
-        <v>1750</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="6" spans="2:6" ht="17" thickBot="1" x14ac:dyDescent="0.25">
@@ -2684,8 +2725,8 @@
         <v>26</v>
       </c>
       <c r="C10" s="13">
-        <f>C18+C4</f>
-        <v>-11.93522783777772</v>
+        <f>C27+C4</f>
+        <v>-14.889328594431133</v>
       </c>
       <c r="D10" s="13"/>
       <c r="E10" s="13"/>
@@ -2701,7 +2742,7 @@
       </c>
       <c r="C12">
         <f>C5+273.15</f>
-        <v>2023.15</v>
+        <v>1273.1500000000001</v>
       </c>
       <c r="F12" s="24"/>
     </row>
@@ -2734,319 +2775,319 @@
     </row>
     <row r="16" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B16" s="18" t="s">
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="C16">
-        <f>('Equilibrium Parameters'!B3/$C$12)+'Equilibrium Parameters'!C3+(('Equilibrium Parameters'!D3*($C$6-1))/C$12)</f>
-        <v>-7.1584402293453273</v>
+        <f>('Equilibrium Parameters'!B13/$C$12)+'Equilibrium Parameters'!C13+(('Equilibrium Parameters'!D13*($C$6-1))/C$12)</f>
+        <v>-5.6970981424026998</v>
       </c>
       <c r="E16" t="s">
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="F16" s="19">
-        <f>$C$10-C16</f>
-        <v>-4.776787608432393</v>
+        <f t="shared" ref="F16:F29" si="0">$C$10-C16</f>
+        <v>-9.1922304520284328</v>
       </c>
     </row>
     <row r="17" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B17" s="18" t="s">
-        <v>5</v>
+        <v>14</v>
       </c>
       <c r="C17">
-        <f>('Equilibrium Parameters'!B4/$C$12)+'Equilibrium Parameters'!C4+(('Equilibrium Parameters'!D4*($C$6-1))/C$12)</f>
-        <v>-7.0995033487383532</v>
+        <f>('Equilibrium Parameters'!B14/$C$12)+'Equilibrium Parameters'!C14+(('Equilibrium Parameters'!D14*($C$6-1))/C$12)</f>
+        <v>-5.322284687585908</v>
       </c>
       <c r="E17" t="s">
-        <v>5</v>
+        <v>14</v>
       </c>
       <c r="F17" s="19">
-        <f t="shared" ref="F17:F32" si="0">$C$10-C17</f>
-        <v>-4.8357244890393671</v>
+        <f t="shared" si="0"/>
+        <v>-9.5670439068452247</v>
       </c>
     </row>
     <row r="18" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B18" s="18" t="s">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="C18">
-        <f>('Equilibrium Parameters'!B5/$C$12)+'Equilibrium Parameters'!C5+(('Equilibrium Parameters'!D5*($C$6-1))/C$12)</f>
-        <v>-6.8852278377777214</v>
+        <f>('Equilibrium Parameters'!B15/$C$12)+'Equilibrium Parameters'!C15+(('Equilibrium Parameters'!D15*($C$6-1))/C$12)</f>
+        <v>-5.6286237285473</v>
       </c>
       <c r="E18" t="s">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="F18" s="19">
         <f t="shared" si="0"/>
-        <v>-5.0499999999999989</v>
+        <v>-9.2607048658838327</v>
       </c>
     </row>
     <row r="19" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B19" s="18" t="s">
-        <v>29</v>
+        <v>38</v>
       </c>
       <c r="C19">
-        <f>(6.54106+0.0012324*(C6/10000)) + (-28163.6+546.32*(C6/10000)-1.13412*(C6/10000)^2+0.0019274*(C6/10000)^3)/(C5+273.15)</f>
-        <v>-7.3795811381649061</v>
+        <f>(-451020+297.595*C12-14.6586*C12*LN(C12))/(8.31441*C12*LN(10))</f>
+        <v>-8.4335986852380227</v>
       </c>
       <c r="E19" t="s">
-        <v>29</v>
+        <v>38</v>
       </c>
       <c r="F19" s="19">
-        <f>$C$10-C19</f>
-        <v>-4.5556466996128142</v>
-      </c>
-      <c r="G19" s="25" t="s">
-        <v>54</v>
+        <f t="shared" si="0"/>
+        <v>-6.45572990919311</v>
       </c>
     </row>
     <row r="20" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B20" s="18" t="s">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="C20">
-        <f>('Equilibrium Parameters'!B7/$C$12)+'Equilibrium Parameters'!C7+(('Equilibrium Parameters'!D7*($C$6-1))/C$12)</f>
-        <v>-3.2038020907990017</v>
+        <f>('Equilibrium Parameters'!B12/$C$12)+'Equilibrium Parameters'!C12+(('Equilibrium Parameters'!D12*($C$6-1))/C$12)</f>
+        <v>-10.22135333621333</v>
       </c>
       <c r="E20" t="s">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="F20" s="19">
         <f t="shared" si="0"/>
-        <v>-8.7314257469787186</v>
+        <v>-4.6679752582178029</v>
       </c>
     </row>
     <row r="21" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B21" s="18" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="C21">
-        <f>('Equilibrium Parameters'!B8/$C$12)+'Equilibrium Parameters'!C8+(('Equilibrium Parameters'!D8*($C$6-1))/C$12)</f>
-        <v>-6.0511531522625592</v>
+        <f>('Equilibrium Parameters'!B10/$C$12)+'Equilibrium Parameters'!C10+(('Equilibrium Parameters'!D10*($C$6-1))/C$12)</f>
+        <v>-10.435405411773944</v>
       </c>
       <c r="E21" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F21" s="19">
         <f t="shared" si="0"/>
-        <v>-5.8840746855151611</v>
+        <v>-4.4539231826571886</v>
       </c>
     </row>
     <row r="22" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B22" s="18" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="C22">
-        <f>('Equilibrium Parameters'!B9/$C$12)+'Equilibrium Parameters'!C9+(('Equilibrium Parameters'!D9*($C$6-1))/C$12)</f>
-        <v>-4.7320864740627222</v>
+        <f>('Equilibrium Parameters'!B11/$C$12)+'Equilibrium Parameters'!C11+(('Equilibrium Parameters'!D11*($C$6-1))/C$12)</f>
+        <v>-10.976974237128381</v>
       </c>
       <c r="E22" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="F22" s="19">
         <f t="shared" si="0"/>
-        <v>-7.2031413637149981</v>
+        <v>-3.9123543573027515</v>
       </c>
     </row>
     <row r="23" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B23" s="18" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C23">
-        <f>('Equilibrium Parameters'!B10/$C$12)+'Equilibrium Parameters'!C10+(('Equilibrium Parameters'!D10*($C$6-1))/C$12)</f>
-        <v>-2.7322919210142604</v>
+        <f>('Equilibrium Parameters'!B9/$C$12)+'Equilibrium Parameters'!C9+(('Equilibrium Parameters'!D9*($C$6-1))/C$12)</f>
+        <v>-11.817123473274945</v>
       </c>
       <c r="E23" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F23" s="19">
         <f t="shared" si="0"/>
-        <v>-9.2029359167634599</v>
+        <v>-3.0722051211561876</v>
       </c>
     </row>
     <row r="24" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B24" s="18" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="C24">
-        <f>('Equilibrium Parameters'!B11/$C$12)+'Equilibrium Parameters'!C11+(('Equilibrium Parameters'!D11*($C$6-1))/C$12)</f>
-        <v>-3.6695671354076556</v>
+        <f>('Equilibrium Parameters'!B7/$C$12)+'Equilibrium Parameters'!C7+(('Equilibrium Parameters'!D7*($C$6-1))/C$12)</f>
+        <v>-12.75636979146212</v>
       </c>
       <c r="E24" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="F24" s="19">
         <f t="shared" si="0"/>
-        <v>-8.2656607023700648</v>
+        <v>-2.1329588029690125</v>
       </c>
     </row>
     <row r="25" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B25" s="18" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="C25">
-        <f>('Equilibrium Parameters'!B12/$C$12)+'Equilibrium Parameters'!C12+(('Equilibrium Parameters'!D12*($C$6-1))/C$12)</f>
-        <v>-2.9623685836443165</v>
+        <f>('Equilibrium Parameters'!B8/$C$12)+'Equilibrium Parameters'!C8+(('Equilibrium Parameters'!D8*($C$6-1))/C$12)</f>
+        <v>-14.405129403448138</v>
       </c>
       <c r="E25" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="F25" s="19">
         <f t="shared" si="0"/>
-        <v>-8.9728592541334038</v>
+        <v>-0.48419919098299502</v>
       </c>
     </row>
     <row r="26" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B26" s="18" t="s">
-        <v>13</v>
+        <v>46</v>
       </c>
       <c r="C26">
-        <f>('Equilibrium Parameters'!B13/$C$12)+'Equilibrium Parameters'!C13+(('Equilibrium Parameters'!D13*($C$6-1))/C$12)</f>
-        <v>1.7271282406148831</v>
+        <f>LOG(EXP((-580563+173*C12)/(8.314*C12)))</f>
+        <v>-14.783207813079107</v>
       </c>
       <c r="E26" t="s">
-        <v>13</v>
+        <v>46</v>
       </c>
       <c r="F26" s="19">
         <f t="shared" si="0"/>
-        <v>-13.662356078392603</v>
+        <v>-0.10612078135202552</v>
+      </c>
+      <c r="G26" s="25" t="s">
+        <v>52</v>
       </c>
     </row>
     <row r="27" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B27" s="18" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="C27">
-        <f>('Equilibrium Parameters'!B14/$C$12)+'Equilibrium Parameters'!C14+(('Equilibrium Parameters'!D14*($C$6-1))/C$12)</f>
-        <v>2.3800426315399275</v>
+        <f>('Equilibrium Parameters'!B5/$C$12)+'Equilibrium Parameters'!C5+(('Equilibrium Parameters'!D5*($C$6-1))/C$12)</f>
+        <v>-14.889328594431133</v>
       </c>
       <c r="E27" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="F27" s="19">
         <f t="shared" si="0"/>
-        <v>-14.315270469317648</v>
+        <v>0</v>
       </c>
     </row>
     <row r="28" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B28" s="18" t="s">
-        <v>15</v>
+        <v>29</v>
       </c>
       <c r="C28">
-        <f>('Equilibrium Parameters'!B15/$C$12)+'Equilibrium Parameters'!C15+(('Equilibrium Parameters'!D15*($C$6-1))/C$12)</f>
-        <v>1.8547402318167219</v>
+        <f>(6.54106+0.0012324*(C6/10000)) + (-28163.6+546.32*(C6/10000)-1.13412*(C6/10000)^2+0.0019274*(C6/10000)^3)/(C5+273.15)</f>
+        <v>-15.580092425957922</v>
       </c>
       <c r="E28" t="s">
-        <v>15</v>
+        <v>29</v>
       </c>
       <c r="F28" s="19">
         <f t="shared" si="0"/>
-        <v>-13.789968069594442</v>
+        <v>0.69076383152678922</v>
+      </c>
+      <c r="G28" s="25" t="s">
+        <v>53</v>
       </c>
     </row>
     <row r="29" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B29" s="18" t="s">
-        <v>28</v>
+        <v>4</v>
       </c>
       <c r="C29">
-        <f>(1/C12*0.4343*120*((0.00251*(C6/10000)^3-0.20044*(C6/10000)^2+10.32257*(C6/10000))-(0.00251*0.0001^3-0.20044*0.0001^2+10.32257*0.0001)))+(LOG(EXP((-911336+212.2423*C12-4.512*C12*LOG(C12))/(8.314*C12))))</f>
-        <v>-13.22255328782814</v>
+        <f>('Equilibrium Parameters'!B3/$C$12)+'Equilibrium Parameters'!C3+(('Equilibrium Parameters'!D3*($C$6-1))/C$12)</f>
+        <v>-15.729370734006205</v>
       </c>
       <c r="E29" t="s">
-        <v>28</v>
+        <v>4</v>
       </c>
       <c r="F29" s="19">
         <f t="shared" si="0"/>
-        <v>1.2873254500504192</v>
+        <v>0.8400421395750719</v>
       </c>
     </row>
     <row r="30" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B30" s="18" t="s">
-        <v>33</v>
+        <v>5</v>
       </c>
       <c r="C30">
-        <f>(-20586/C12) - 0.044 +LOG10(C6/10000) - 0.028 * ((C6/10000)-1)/C12</f>
-        <v>-14.219207969157008</v>
+        <f>('Equilibrium Parameters'!B4/$C$12)+'Equilibrium Parameters'!C4+(('Equilibrium Parameters'!D4*($C$6-1))/C$12)</f>
+        <v>-15.695212818599533</v>
       </c>
       <c r="E30" t="s">
-        <v>33</v>
+        <v>5</v>
       </c>
       <c r="F30" s="19">
-        <f t="shared" si="0"/>
-        <v>2.2839801313792876</v>
+        <f t="shared" ref="F30:F32" si="1">$C$10-C30</f>
+        <v>0.80588422416840011</v>
       </c>
     </row>
     <row r="31" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B31" s="18" t="s">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="C31">
-        <f>(-451020+297.595*C12-14.6586*C12*LN(C12))/(8.31441*C12*LN(10))</f>
-        <v>-1.9285755343579587</v>
+        <f>(-20586/C12) - 0.044 +LOG10(C6) - 0.028 * ((C6)-1)/C12</f>
+        <v>-16.213343753681812</v>
       </c>
       <c r="E31" t="s">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="F31" s="19">
-        <f t="shared" si="0"/>
-        <v>-10.006652303419761</v>
+        <f t="shared" si="1"/>
+        <v>1.3240151592506795</v>
       </c>
     </row>
     <row r="32" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B32" s="18" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C32">
         <f>LOG(EXP((-758585+349.718*C12-25.5216*C12*LN(C12)+0.00935*C12^2)/(8.314*C12)))</f>
-        <v>-10.478588792111982</v>
+        <v>-21.765471947809271</v>
       </c>
       <c r="E32" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="F32" s="19">
-        <f t="shared" si="0"/>
-        <v>-1.4566390456657388</v>
+        <f t="shared" si="1"/>
+        <v>6.8761433533781382</v>
       </c>
       <c r="G32" s="25" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="33" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B33" s="18" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="C33">
-        <f>LOG(EXP((-580563+173*C12)/(8.314*C12)))</f>
-        <v>-5.9528713663148674</v>
+        <f>2*LOG(EXP((-376969-4.19123*C12+10.02409*C12*LN(C12))/(8.314*C12)))</f>
+        <v>-23.884430305504146</v>
       </c>
       <c r="E33" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="F33" s="19">
         <f>$C$10-C33</f>
-        <v>-5.982356471462853</v>
+        <v>8.9951017110730138</v>
       </c>
       <c r="G33" s="25" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="34" spans="2:7" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B34" s="20" t="s">
-        <v>50</v>
+        <v>28</v>
       </c>
       <c r="C34" s="21">
-        <f>2*LOG(EXP((-376969-4.19123*C12+10.02409*C12*LN(C12))/(8.314*C12)))</f>
-        <v>-11.932023421684903</v>
+        <f>(1/C12*0.4343*120*((0.00251*(C6/10000)^3-0.20044*(C6/10000)^2+10.32257*(C6/10000))-(0.00251*0.0001^3-0.20044*0.0001^2+10.32257*0.0001)))+(LOG(EXP((-911336+212.2423*C12-4.512*C12*LOG(C12))/(8.314*C12))))</f>
+        <v>-27.036522869930032</v>
       </c>
       <c r="D34" s="21"/>
       <c r="E34" s="21" t="s">
-        <v>50</v>
+        <v>28</v>
       </c>
       <c r="F34" s="22">
         <f>$C$10-C34</f>
-        <v>-3.2044160928172971E-3</v>
-      </c>
-      <c r="G34" s="25" t="s">
-        <v>53</v>
+        <v>12.147194275498899</v>
       </c>
     </row>
   </sheetData>
@@ -3059,12 +3100,12 @@
   <dimension ref="A1:D39"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="12" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.2">
@@ -3262,7 +3303,7 @@
         <v>29</v>
       </c>
       <c r="B18" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.2">
@@ -3280,82 +3321,82 @@
         <v>33</v>
       </c>
       <c r="B22" t="s">
-        <v>34</v>
+        <v>68</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A25" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B25" t="s">
         <v>37</v>
-      </c>
-      <c r="B25" t="s">
-        <v>38</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A28" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="B28" t="s">
         <v>40</v>
-      </c>
-      <c r="B28" t="s">
-        <v>41</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A32" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B32" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A35" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="B35" t="s">
         <v>47</v>
-      </c>
-      <c r="B35" t="s">
-        <v>48</v>
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A38" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="B38" t="s">
         <v>50</v>
-      </c>
-      <c r="B38" t="s">
-        <v>51</v>
       </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
   </sheetData>
@@ -3367,72 +3408,77 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9FC30CFD-6A9F-0E42-88FD-691A50553FEB}">
-  <dimension ref="A1:A14"/>
+  <dimension ref="A1:A15"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A1" s="26" t="s">
-        <v>68</v>
+    <row r="1" spans="1:1" ht="21" x14ac:dyDescent="0.25">
+      <c r="A1" s="27" t="s">
+        <v>69</v>
       </c>
     </row>
     <row r="2" spans="1:1" ht="20" x14ac:dyDescent="0.2">
-      <c r="A2" s="27" t="s">
+      <c r="A2" s="26" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" ht="20" x14ac:dyDescent="0.2">
+      <c r="A3" s="26" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" ht="20" x14ac:dyDescent="0.2">
+      <c r="A4" s="26" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" ht="20" x14ac:dyDescent="0.2">
+      <c r="A5" s="26" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" ht="20" x14ac:dyDescent="0.2">
+      <c r="A6" s="26" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" ht="20" x14ac:dyDescent="0.2">
+      <c r="A7" s="26" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1" ht="20" x14ac:dyDescent="0.2">
+      <c r="A9" s="26" t="s">
         <v>59</v>
-      </c>
-    </row>
-    <row r="3" spans="1:1" ht="20" x14ac:dyDescent="0.2">
-      <c r="A3" s="27" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="4" spans="1:1" ht="20" x14ac:dyDescent="0.2">
-      <c r="A4" s="27" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="5" spans="1:1" ht="20" x14ac:dyDescent="0.2">
-      <c r="A5" s="27" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="6" spans="1:1" ht="20" x14ac:dyDescent="0.2">
-      <c r="A6" s="27" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="8" spans="1:1" ht="20" x14ac:dyDescent="0.2">
-      <c r="A8" s="27" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A9" t="s">
-        <v>61</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>65</v>
+        <v>60</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="14" spans="1:1" ht="17" x14ac:dyDescent="0.2">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="14" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>63</v>
+      </c>
+    </row>
+    <row r="15" spans="1:1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
+        <v>62</v>
       </c>
     </row>
   </sheetData>

</xml_diff>